<commit_message>
Reorganize QA test case library
- restructure test cases into API, Authentication, BibleReading, CommunitySystem, and DB folders

- add leader notification bug report artifacts and refresh supporting bug report docs

- update notification coverage workbooks and validation assets for cleaner QA navigation
</commit_message>
<xml_diff>
--- a/qa-docs/test-cases/Done/Me/Notifications/VerseByVerse_Notifications_Security_Test_Cases.xlsx
+++ b/qa-docs/test-cases/Done/Me/Notifications/VerseByVerse_Notifications_Security_Test_Cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\versebyverse-quality-engineering\qa-docs\test-cases\Notifications\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\versebyverse-quality-engineering\qa-docs\test-cases\Done\Me\Notifications\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6998648E-3471-4408-8DE2-D91A85E3836F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C8ED50-3824-4FCE-BA73-766CFADB5B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29970" yWindow="5325" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -61,9 +61,6 @@
     <t>High</t>
   </si>
   <si>
-    <t>Not Run</t>
-  </si>
-  <si>
     <t>Security</t>
   </si>
   <si>
@@ -543,6 +540,9 @@
   </si>
   <si>
     <t>VerseByVerse -  Notifications Security Test Cases</t>
+  </si>
+  <si>
+    <t>Passed</t>
   </si>
 </sst>
 </file>
@@ -932,7 +932,7 @@
     <col min="5" max="5" width="31.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="35.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="73.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="68.140625" customWidth="1"/>
     <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
@@ -940,7 +940,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -990,877 +990,877 @@
     </row>
     <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="I3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="I4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="I5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="I6" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="I7" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="I8" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="I9" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>64</v>
-      </c>
       <c r="I10" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H11" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="I11" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="H12" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="I12" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>82</v>
-      </c>
       <c r="I13" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>88</v>
-      </c>
       <c r="I14" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>94</v>
-      </c>
       <c r="I15" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="H16" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>99</v>
-      </c>
       <c r="I16" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="H17" s="2" t="s">
-        <v>105</v>
-      </c>
       <c r="I17" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="I18" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="G19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="G19" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>115</v>
-      </c>
       <c r="I19" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="F20" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="G20" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="H20" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>121</v>
-      </c>
       <c r="I20" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="E21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="J21" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="F22" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="H22" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="H22" s="2" t="s">
-        <v>132</v>
-      </c>
       <c r="I22" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="H23" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="H23" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="I23" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="E24" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="I24" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="J24" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" s="2" t="s">
+      <c r="E25" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="G25" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="H25" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="H25" s="2" t="s">
-        <v>149</v>
-      </c>
       <c r="I25" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D26" s="2" t="s">
+      <c r="E26" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="H26" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="H26" s="2" t="s">
-        <v>155</v>
-      </c>
       <c r="I26" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27" s="2" t="s">
+      <c r="E27" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="F27" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="G27" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="H27" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="H27" s="2" t="s">
-        <v>161</v>
-      </c>
       <c r="I27" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -1868,6 +1868,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1:K1048576" xr:uid="{D5918E79-C35A-4870-A859-EE2E0CEE220B}">
+      <formula1>"Passed,Failed,Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>